<commit_message>
add top5% of R32 opponents with %
</commit_message>
<xml_diff>
--- a/data/raw/football/matches_grouprounds.xlsx
+++ b/data/raw/football/matches_grouprounds.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jongdjj\Documents\VSCode\Playground_local\data\raw\football\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jongdjj\Documents\VSCode\football_WC2026\data\raw\football\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E29CFB3-B436-48C3-9BE1-0C6C745ACA57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83EC3851-4511-43C6-8F0B-C8E7FD3FE9C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="298" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="122">
   <si>
     <t>id</t>
   </si>
@@ -380,6 +380,12 @@
   </si>
   <si>
     <t>4-0</t>
+  </si>
+  <si>
+    <t>3-2</t>
+  </si>
+  <si>
+    <t>1-2</t>
   </si>
 </sst>
 </file>
@@ -2114,6 +2120,9 @@
       <c r="I42">
         <v>2</v>
       </c>
+      <c r="J42" s="4" t="s">
+        <v>102</v>
+      </c>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A43">
@@ -2143,6 +2152,9 @@
       <c r="I43">
         <v>2</v>
       </c>
+      <c r="J43" s="4" t="s">
+        <v>114</v>
+      </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A44">
@@ -2172,6 +2184,9 @@
       <c r="I44">
         <v>2</v>
       </c>
+      <c r="J44" s="4" t="s">
+        <v>120</v>
+      </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A45">
@@ -2200,6 +2215,9 @@
       </c>
       <c r="I45">
         <v>2</v>
+      </c>
+      <c r="J45" s="4" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.3">

</xml_diff>